<commit_message>
Minor fixes and additional assets
</commit_message>
<xml_diff>
--- a/Documents/Character List by Class.xlsx
+++ b/Documents/Character List by Class.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hugob\BindingStories\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4D0D02D-887A-4D05-8433-A28E743912E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCE8EC73-928B-4C51-8110-C24733B41E83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="205">
   <si>
     <t>Class</t>
   </si>
@@ -637,6 +637,9 @@
   </si>
   <si>
     <t>Ritsu</t>
+  </si>
+  <si>
+    <t>Cid</t>
   </si>
 </sst>
 </file>
@@ -957,7 +960,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E181"/>
+  <dimension ref="A1:E182"/>
   <sheetFormatPr defaultColWidth="15.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.21875" style="1" customWidth="1"/>
@@ -1654,209 +1657,209 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B73" s="1" t="s">
-        <v>142</v>
+        <v>204</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="D73" s="1">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B74" s="1" t="s">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C74" s="1" t="s">
         <v>44</v>
       </c>
       <c r="D74" s="1">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B75" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D75" s="1">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B76" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="C75" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D75" s="1">
+      <c r="C76" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D76" s="1">
         <v>25</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A77" s="1" t="s">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A78" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B77" s="1" t="s">
+      <c r="B78" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C77" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D77" s="1">
+      <c r="C78" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D78" s="1">
         <v>3</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B78" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="C78" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D78" s="1">
-        <v>12</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B79" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="D79" s="1">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B80" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D80" s="1">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B81" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C80" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D80" s="1">
+      <c r="C81" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D81" s="1">
         <v>21</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A82" s="1" t="s">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A83" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B82" s="1" t="s">
+      <c r="B83" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C82" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D82" s="1">
+      <c r="C83" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D83" s="1">
         <v>2</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B83" s="1" t="s">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B84" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="C83" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D83" s="1">
+      <c r="C84" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D84" s="1">
         <v>9</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A85" s="1" t="s">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A86" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B85" s="1" t="s">
+      <c r="B86" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C85" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D85" s="1">
+      <c r="C86" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D86" s="1">
         <v>12</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B86" s="1" t="s">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B87" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="C86" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D86" s="1">
+      <c r="C87" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D87" s="1">
         <v>17</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A88" s="1" t="s">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A89" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B88" s="1" t="s">
+      <c r="B89" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C88" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D88" s="1">
+      <c r="C89" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D89" s="1">
         <v>14</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B89" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C89" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D89" s="1">
-        <v>25</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B90" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D90" s="1">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B91" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C90" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D90" s="1">
+      <c r="C91" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D91" s="1">
         <v>34</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A92" s="1" t="s">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A93" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B92" s="1" t="s">
+      <c r="B93" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C92" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D92" s="1">
+      <c r="C93" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D93" s="1">
         <v>2</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B93" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="C93" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D93" s="1">
-        <v>10</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B94" s="1" t="s">
-        <v>148</v>
+        <v>85</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="D94" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B95" s="1" t="s">
-        <v>114</v>
+        <v>148</v>
       </c>
       <c r="C95" s="1" t="s">
         <v>44</v>
@@ -1867,466 +1870,466 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B96" s="1" t="s">
-        <v>164</v>
+        <v>114</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>44</v>
       </c>
       <c r="D96" s="1">
-        <v>26</v>
+        <v>15</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B97" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D97" s="1">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B98" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="C97" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D97" s="1">
+      <c r="C98" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D98" s="1">
         <v>31</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A99" s="1" t="s">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A100" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B99" s="1" t="s">
+      <c r="B100" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C99" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D99" s="1">
+      <c r="C100" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D100" s="1">
         <v>4</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B100" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="C100" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D100" s="1">
-        <v>12</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B101" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D101" s="1">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B102" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="C101" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D101" s="1">
+      <c r="C102" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D102" s="1">
         <v>33</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A103" s="1" t="s">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A104" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="B103" s="1" t="s">
+      <c r="B104" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="C103" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D103" s="1">
+      <c r="C104" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D104" s="1">
         <v>9</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B104" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="C104" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D104" s="1">
-        <v>22</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B105" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D105" s="1">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B106" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="C105" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D105" s="1">
+      <c r="C106" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D106" s="1">
         <v>25</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A107" s="1" t="s">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A108" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B107" s="1" t="s">
+      <c r="B108" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C107" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D107" s="1">
+      <c r="C108" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D108" s="1">
         <v>3</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B108" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="C108" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D108" s="1">
-        <v>6</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B109" s="1" t="s">
-        <v>172</v>
+        <v>152</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D109" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B110" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D110" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B111" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C110" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D110" s="1">
+      <c r="C111" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D111" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A112" s="1" t="s">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A113" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B112" s="1" t="s">
+      <c r="B113" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C112" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D112" s="1">
+      <c r="C113" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D113" s="1">
         <v>3</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B113" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="C113" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D113" s="1">
-        <v>8</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B114" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D114" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B115" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="C114" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D114" s="1">
+      <c r="C115" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D115" s="1">
         <v>16</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A116" s="1" t="s">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A117" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B116" s="1" t="s">
+      <c r="B117" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C116" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D116" s="1">
+      <c r="C117" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D117" s="1">
         <v>9</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B117" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="C117" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D117" s="1">
-        <v>17</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B118" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D118" s="1">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B119" s="1" t="s">
-        <v>91</v>
+        <v>169</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D119" s="1">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B120" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D120" s="1">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B121" s="1" t="s">
-        <v>146</v>
+        <v>90</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D121" s="1">
-        <v>32</v>
+        <v>22</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B122" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C122" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D122" s="1">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B123" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D123" s="1">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B124" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="C123" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D123" s="1">
+      <c r="C124" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D124" s="1">
         <v>39</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A125" s="1" t="s">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A126" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B125" s="1" t="s">
+      <c r="B126" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C125" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D125" s="1">
+      <c r="C126" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D126" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B126" s="1" t="s">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B127" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="C126" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D126" s="1">
+      <c r="C127" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D127" s="1">
         <v>17</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A128" s="1" t="s">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A129" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B128" s="1" t="s">
+      <c r="B129" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C128" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D128" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B129" s="1" t="s">
-        <v>180</v>
-      </c>
       <c r="C129" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D129" s="1">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B130" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C130" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D130" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B131" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="C130" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D130" s="1">
+      <c r="C131" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D131" s="1">
         <v>23</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A132" s="1" t="s">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A133" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B132" s="1" t="s">
+      <c r="B133" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C132" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D132" s="1">
+      <c r="C133" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D133" s="1">
         <v>17</v>
-      </c>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B133" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C133" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D133" s="1">
-        <v>18</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B134" s="1" t="s">
-        <v>161</v>
+        <v>96</v>
       </c>
       <c r="C134" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D134" s="1">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B135" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C135" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D135" s="1">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B136" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="C135" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D135" s="1" t="s">
+      <c r="C136" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D136" s="1" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A137" s="1" t="s">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A138" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B137" s="1" t="s">
+      <c r="B138" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C137" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D137" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B138" s="1" t="s">
-        <v>98</v>
-      </c>
       <c r="C138" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D138" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B139" s="1" t="s">
-        <v>195</v>
+        <v>98</v>
       </c>
       <c r="C139" s="1" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="D139" s="1">
-        <v>26</v>
+        <v>7</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B140" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="C140" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D140" s="1">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B141" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C140" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D140" s="1">
+      <c r="C141" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D141" s="1">
         <v>27</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A142" s="1" t="s">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A143" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="B142" s="1" t="s">
+      <c r="B143" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C142" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D142" s="1">
+      <c r="C143" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D143" s="1">
         <v>2</v>
-      </c>
-    </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B143" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="C143" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D143" s="1">
-        <v>9</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B144" s="1" t="s">
-        <v>102</v>
+        <v>190</v>
       </c>
       <c r="C144" s="1" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="D144" s="1">
-        <v>27</v>
+        <v>9</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B145" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>44</v>
@@ -2335,236 +2338,230 @@
         <v>27</v>
       </c>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A147" s="1" t="s">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B146" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C146" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D146" s="1">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A148" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B147" s="1" t="s">
+      <c r="B148" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C147" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D147" s="1">
+      <c r="C148" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D148" s="1">
         <v>7</v>
-      </c>
-    </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B148" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="C148" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D148" s="1">
-        <v>27</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B149" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C149" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D149" s="1">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B150" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="C149" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D149" s="1">
+      <c r="C150" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D150" s="1">
         <v>33</v>
       </c>
     </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A151" s="1" t="s">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A152" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B151" s="1" t="s">
+      <c r="B152" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="C151" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D151" s="1">
+      <c r="C152" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D152" s="1">
         <v>18</v>
-      </c>
-    </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B152" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C152" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D152" s="1">
-        <v>23</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B153" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C153" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D153" s="1">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B154" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="C153" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D153" s="1">
+      <c r="C154" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D154" s="1">
         <v>31</v>
       </c>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A155" s="1" t="s">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A156" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B155" s="1" t="s">
+      <c r="B156" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="C155" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D155" s="1">
+      <c r="C156" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D156" s="1">
         <v>3</v>
-      </c>
-    </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B156" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="C156" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D156" s="1">
-        <v>6</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B157" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C157" s="1" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="D157" s="1">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B158" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C158" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D158" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B159" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="C158" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D158" s="1">
+      <c r="C159" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D159" s="1">
         <v>26</v>
       </c>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A160" s="1" t="s">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A161" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B160" s="1" t="s">
+      <c r="B161" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C160" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D160" s="1">
+      <c r="C161" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D161" s="1">
         <v>5</v>
-      </c>
-    </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B161" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="C161" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D161" s="1">
-        <v>6</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B162" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C162" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D162" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B163" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C162" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D162" s="1">
+      <c r="C163" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D163" s="1">
         <v>8</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A164" s="1" t="s">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A165" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B164" s="1" t="s">
+      <c r="B165" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C164" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D164" s="1">
+      <c r="C165" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D165" s="1">
         <v>4</v>
-      </c>
-    </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B165" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="C165" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D165" s="1">
-        <v>11</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B166" s="1" t="s">
-        <v>162</v>
+        <v>137</v>
       </c>
       <c r="C166" s="1" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="D166" s="1">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B167" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C167" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D167" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B168" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="C167" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D167" s="1">
+      <c r="C168" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D168" s="1">
         <v>24</v>
-      </c>
-    </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A169" s="1" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A170" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="B170" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="C170" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D170" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="E170" s="1" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A171" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C171" s="1" t="s">
         <v>6</v>
@@ -2573,117 +2570,134 @@
         <v>173</v>
       </c>
       <c r="E171" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A172" s="1" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B172" s="1" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="C172" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D172" s="1">
-        <v>8</v>
+      <c r="D172" s="1" t="s">
+        <v>173</v>
       </c>
       <c r="E172" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A173" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B173" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C173" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D173" s="1">
+        <v>8</v>
+      </c>
+      <c r="E173" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A174" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B173" s="1" t="s">
+      <c r="B174" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="C173" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D173" s="1">
+      <c r="C174" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D174" s="1">
         <v>4</v>
       </c>
-      <c r="E173" s="1" t="s">
+      <c r="E174" s="1" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B174" s="1" t="s">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B175" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="C174" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D174" s="1">
+      <c r="C175" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D175" s="1">
         <v>27</v>
-      </c>
-    </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A175" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B175" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="C175" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D175" s="1">
-        <v>12</v>
-      </c>
-      <c r="E175" s="1" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A176" s="1" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="B176" s="1" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C176" s="1" t="s">
         <v>44</v>
       </c>
       <c r="D176" s="1">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E176" s="1" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A177" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B177" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C177" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D177" s="1">
+        <v>1</v>
+      </c>
+      <c r="E177" s="1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A178" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="B177" s="1" t="s">
+      <c r="B178" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="C177" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D177" s="1">
+      <c r="C178" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D178" s="1">
         <v>25</v>
       </c>
-      <c r="E177" s="1" t="s">
+      <c r="E178" s="1" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A179" s="1" t="s">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A180" s="1" t="s">
         <v>138</v>
-      </c>
-    </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B180" s="1" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B181" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B182" s="1" t="s">
         <v>140</v>
       </c>
     </row>

</xml_diff>

<commit_message>
What a month of forgetting to commit does (3800 files)
</commit_message>
<xml_diff>
--- a/Documents/Character List by Class.xlsx
+++ b/Documents/Character List by Class.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hugob\BindingStories\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCE8EC73-928B-4C51-8110-C24733B41E83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F945299-EA54-46F0-B49B-E83CE9C13509}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="200">
   <si>
     <t>Class</t>
   </si>
@@ -577,21 +577,6 @@
   </si>
   <si>
     <t>Vega</t>
-  </si>
-  <si>
-    <t>Effris</t>
-  </si>
-  <si>
-    <t>Destio</t>
-  </si>
-  <si>
-    <t>Dancer</t>
-  </si>
-  <si>
-    <t>Asty</t>
-  </si>
-  <si>
-    <t>-</t>
   </si>
   <si>
     <t>Kettei</t>
@@ -960,7 +945,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E182"/>
+  <dimension ref="A1:E179"/>
   <sheetFormatPr defaultColWidth="15.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.21875" style="1" customWidth="1"/>
@@ -1004,7 +989,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
@@ -1040,7 +1025,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>6</v>
@@ -1148,7 +1133,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B19" s="1" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>44</v>
@@ -1220,7 +1205,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B27" s="1" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>44</v>
@@ -1450,7 +1435,7 @@
         <v>21</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>51</v>
@@ -1461,7 +1446,7 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B53" s="1" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>51</v>
@@ -1657,7 +1642,7 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B73" s="1" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>6</v>
@@ -1688,178 +1673,178 @@
         <v>18</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B76" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="C76" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D76" s="1">
-        <v>25</v>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A77" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D77" s="1">
+        <v>3</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A78" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="B78" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C78" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D78" s="1">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B79" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="D79" s="1">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B80" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>44</v>
       </c>
       <c r="D80" s="1">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B81" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="C81" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D81" s="1">
         <v>21</v>
       </c>
     </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A82" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D82" s="1">
+        <v>2</v>
+      </c>
+    </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A83" s="1" t="s">
+      <c r="B83" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D83" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A85" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D85" s="1">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B86" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D86" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A88" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D88" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B89" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D89" s="1">
         <v>25</v>
-      </c>
-      <c r="B83" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C83" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D83" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B84" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D84" s="1">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A86" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B86" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C86" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D86" s="1">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B87" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="C87" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D87" s="1">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A89" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B89" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C89" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D89" s="1">
-        <v>14</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B90" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D90" s="1">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B91" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="C91" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D91" s="1">
         <v>34</v>
       </c>
     </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A92" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D92" s="1">
+        <v>2</v>
+      </c>
+    </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A93" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="B93" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C93" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D93" s="1">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B94" s="1" t="s">
-        <v>85</v>
+        <v>148</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="D94" s="1">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B95" s="1" t="s">
-        <v>148</v>
+        <v>114</v>
       </c>
       <c r="C95" s="1" t="s">
         <v>44</v>
@@ -1870,834 +1855,795 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B96" s="1" t="s">
-        <v>114</v>
+        <v>164</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>44</v>
       </c>
       <c r="D96" s="1">
-        <v>15</v>
+        <v>26</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B97" s="1" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C97" s="1" t="s">
         <v>44</v>
       </c>
       <c r="D97" s="1">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B98" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="C98" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D98" s="1">
         <v>31</v>
       </c>
     </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A99" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D99" s="1">
+        <v>4</v>
+      </c>
+    </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A100" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="B100" s="1" t="s">
-        <v>86</v>
+        <v>157</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="D100" s="1">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B101" s="1" t="s">
-        <v>157</v>
+        <v>195</v>
       </c>
       <c r="C101" s="1" t="s">
         <v>44</v>
       </c>
       <c r="D101" s="1">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B102" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="C102" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D102" s="1">
         <v>33</v>
       </c>
     </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A103" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D103" s="1">
+        <v>9</v>
+      </c>
+    </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A104" s="1" t="s">
-        <v>174</v>
-      </c>
       <c r="B104" s="1" t="s">
-        <v>176</v>
+        <v>133</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="D104" s="1">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B105" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="C105" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D105" s="1">
         <v>22</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A106" s="1" t="s">
+        <v>30</v>
+      </c>
       <c r="B106" s="1" t="s">
-        <v>185</v>
+        <v>87</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="D106" s="1">
-        <v>25</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B107" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D107" s="1">
+        <v>7</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A108" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="B108" s="1" t="s">
-        <v>87</v>
+        <v>166</v>
       </c>
       <c r="C108" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D108" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A110" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D110" s="1">
         <v>3</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B109" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="C109" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D109" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B110" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="C110" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D110" s="1">
-        <v>7</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B111" s="1" t="s">
-        <v>166</v>
+        <v>134</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D111" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A113" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B113" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C113" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D113" s="1">
-        <v>3</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B112" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D112" s="1">
+        <v>16</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A114" s="1" t="s">
+        <v>32</v>
+      </c>
       <c r="B114" s="1" t="s">
-        <v>134</v>
+        <v>89</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D114" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B115" s="1" t="s">
-        <v>143</v>
+        <v>170</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D115" s="1">
-        <v>16</v>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B116" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D116" s="1">
+        <v>19</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A117" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="B117" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D117" s="1">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B118" s="1" t="s">
-        <v>170</v>
+        <v>90</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D118" s="1">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B119" s="1" t="s">
-        <v>169</v>
+        <v>146</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D119" s="1">
-        <v>19</v>
+        <v>32</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B120" s="1" t="s">
-        <v>91</v>
+        <v>147</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D120" s="1">
-        <v>20</v>
+        <v>36</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B121" s="1" t="s">
-        <v>90</v>
+        <v>167</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D121" s="1">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B122" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="C122" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D122" s="1">
-        <v>32</v>
+        <v>39</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A123" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="B123" s="1" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="C123" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D123" s="1">
-        <v>36</v>
+        <v>6</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B124" s="1" t="s">
-        <v>167</v>
+        <v>92</v>
       </c>
       <c r="C124" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D124" s="1">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A126" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B126" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C126" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D126" s="1">
         <v>10</v>
       </c>
     </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B125" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C125" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D125" s="1">
+        <v>17</v>
+      </c>
+    </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A127" s="1" t="s">
+        <v>34</v>
+      </c>
       <c r="B127" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C127" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D127" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B128" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C128" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D128" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B129" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C129" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D129" s="1">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A131" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C131" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D131" s="1">
         <v>17</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A129" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B129" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="C129" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D129" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B130" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="C130" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D130" s="1">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B131" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="C131" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D131" s="1">
-        <v>23</v>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B132" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C132" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D132" s="1">
+        <v>18</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A133" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="B133" s="1" t="s">
-        <v>95</v>
+        <v>161</v>
       </c>
       <c r="C133" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D133" s="1">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B134" s="1" t="s">
-        <v>96</v>
+        <v>188</v>
       </c>
       <c r="C134" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D134" s="1">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B135" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="C135" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D135" s="1">
-        <v>22</v>
+      <c r="D134" s="1" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A136" s="1" t="s">
+        <v>36</v>
+      </c>
       <c r="B136" s="1" t="s">
-        <v>193</v>
+        <v>97</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D136" s="1" t="s">
-        <v>194</v>
+        <v>6</v>
+      </c>
+      <c r="D136" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B137" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C137" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D137" s="1">
+        <v>7</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A138" s="1" t="s">
-        <v>36</v>
-      </c>
       <c r="B138" s="1" t="s">
-        <v>97</v>
+        <v>190</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="D138" s="1">
-        <v>6</v>
+        <v>26</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B139" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C139" s="1" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="D139" s="1">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B140" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="C140" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D140" s="1">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A141" s="1" t="s">
+        <v>144</v>
+      </c>
       <c r="B141" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="D141" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B142" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C142" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D142" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B143" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C143" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D143" s="1">
         <v>27</v>
-      </c>
-    </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A143" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="B143" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="C143" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D143" s="1">
-        <v>2</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B144" s="1" t="s">
-        <v>190</v>
+        <v>103</v>
       </c>
       <c r="C144" s="1" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="D144" s="1">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B145" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="C145" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D145" s="1">
         <v>27</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A146" s="1" t="s">
+        <v>37</v>
+      </c>
       <c r="B146" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="D146" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B147" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C147" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D147" s="1">
         <v>27</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A148" s="1" t="s">
-        <v>37</v>
-      </c>
       <c r="B148" s="1" t="s">
-        <v>104</v>
+        <v>153</v>
       </c>
       <c r="C148" s="1" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="D148" s="1">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B149" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="C149" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D149" s="1">
-        <v>27</v>
+        <v>33</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A150" s="1" t="s">
+        <v>38</v>
+      </c>
       <c r="B150" s="1" t="s">
-        <v>153</v>
+        <v>105</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="D150" s="1">
-        <v>33</v>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B151" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C151" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D151" s="1">
+        <v>23</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A152" s="1" t="s">
-        <v>38</v>
-      </c>
       <c r="B152" s="1" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="C152" s="1" t="s">
         <v>51</v>
       </c>
       <c r="D152" s="1">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B153" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C153" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D153" s="1">
-        <v>23</v>
+        <v>31</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A154" s="1" t="s">
+        <v>39</v>
+      </c>
       <c r="B154" s="1" t="s">
-        <v>191</v>
+        <v>107</v>
       </c>
       <c r="C154" s="1" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="D154" s="1">
-        <v>31</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B155" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C155" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D155" s="1">
+        <v>6</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A156" s="1" t="s">
-        <v>39</v>
-      </c>
       <c r="B156" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C156" s="1" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="D156" s="1">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B157" s="1" t="s">
-        <v>108</v>
+        <v>145</v>
       </c>
       <c r="C157" s="1" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="D157" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B158" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C158" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D158" s="1">
-        <v>10</v>
+        <v>26</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A159" s="1" t="s">
+        <v>40</v>
+      </c>
       <c r="B159" s="1" t="s">
-        <v>145</v>
+        <v>111</v>
       </c>
       <c r="C159" s="1" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="D159" s="1">
-        <v>26</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B160" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C160" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D160" s="1">
+        <v>6</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A161" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="B161" s="1" t="s">
-        <v>111</v>
+        <v>149</v>
       </c>
       <c r="C161" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D161" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B162" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="C162" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D162" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A163" s="1" t="s">
+        <v>41</v>
+      </c>
       <c r="B163" s="1" t="s">
-        <v>149</v>
+        <v>112</v>
       </c>
       <c r="C163" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D163" s="1">
-        <v>8</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B164" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C164" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D164" s="1">
+        <v>11</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A165" s="1" t="s">
-        <v>41</v>
-      </c>
       <c r="B165" s="1" t="s">
-        <v>112</v>
+        <v>162</v>
       </c>
       <c r="C165" s="1" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="D165" s="1">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B166" s="1" t="s">
-        <v>137</v>
+        <v>113</v>
       </c>
       <c r="C166" s="1" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="D166" s="1">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B167" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="C167" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D167" s="1">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B168" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="C168" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D168" s="1">
-        <v>24</v>
+      <c r="A168" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A169" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B169" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C169" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D169" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="E169" s="1" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A170" s="1" t="s">
-        <v>115</v>
+        <v>119</v>
+      </c>
+      <c r="B170" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C170" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D170" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="E170" s="1" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A171" s="1" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="C171" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D171" s="1" t="s">
-        <v>173</v>
+      <c r="D171" s="1">
+        <v>8</v>
       </c>
       <c r="E171" s="1" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A172" s="1" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="B172" s="1" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="C172" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D172" s="1" t="s">
-        <v>173</v>
+      <c r="D172" s="1">
+        <v>4</v>
       </c>
       <c r="E172" s="1" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A173" s="1" t="s">
-        <v>122</v>
-      </c>
       <c r="B173" s="1" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C173" s="1" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="D173" s="1">
-        <v>8</v>
-      </c>
-      <c r="E173" s="1" t="s">
-        <v>124</v>
+        <v>27</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A174" s="1" t="s">
-        <v>126</v>
+        <v>154</v>
       </c>
       <c r="B174" s="1" t="s">
-        <v>127</v>
+        <v>155</v>
       </c>
       <c r="C174" s="1" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="D174" s="1">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E174" s="1" t="s">
-        <v>129</v>
+        <v>156</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A175" s="1" t="s">
+        <v>158</v>
+      </c>
       <c r="B175" s="1" t="s">
-        <v>128</v>
+        <v>159</v>
       </c>
       <c r="C175" s="1" t="s">
         <v>44</v>
       </c>
       <c r="D175" s="1">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A176" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B176" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="C176" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D176" s="1">
-        <v>12</v>
-      </c>
-      <c r="E176" s="1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="E175" s="1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A177" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="B177" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="C177" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D177" s="1">
-        <v>1</v>
-      </c>
-      <c r="E177" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A178" s="1" t="s">
-        <v>186</v>
-      </c>
+        <v>138</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B178" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="C178" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D178" s="1">
-        <v>25</v>
-      </c>
-      <c r="E178" s="1" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A180" s="1" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B181" s="1" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B182" s="1" t="s">
+    <row r="179" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B179" s="1" t="s">
         <v>140</v>
       </c>
     </row>

</xml_diff>